<commit_message>
Docs and patch copies for the word-pass fixes (weaknesses 1 to 3); trigger list rebuilt
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YEUNXbYb9LDbJLc2ziqL3n
</commit_message>
<xml_diff>
--- a/acts/ACT_TRIGGER_LIST.xlsx
+++ b/acts/ACT_TRIGGER_LIST.xlsx
@@ -508,7 +508,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>I said the word pass had 'four deliberate changes' from the workbook, each required by its own false-positive rules. That was incomplete. This sheet lists them all: some changes make a trigger NARROWER than the workbook (POCSO row 3, the dowry row), several make it LOOSER by dropping the 'nearby context' the workbook required ('undue advantage', 'trap case', 'known sources of income', 'provisional attachment', bare 'laundering', bare 'terror...'), and the Corruption Act's role/verb/money lists are mine.</t>
+          <t>I said the word pass had 'four deliberate changes' from the workbook, each required by its own false-positive rules. That was incomplete. This sheet lists them all: some changes make a trigger NARROWER than the workbook (POCSO row 3, the dowry row), several make it LOOSER by dropping the 'nearby context' the workbook required ('undue advantage', 'trap case', 'known sources of income', 'provisional attachment', bare 'laundering'; the bare 'terror...' and bare 'Enforcement Directorate' rows were tightened again on 2026-10-17), and the Corruption Act's role/verb/money lists are mine.</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -986,7 +986,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>(?:(?:(?:public servant|government (?:officer|official|servant|employee|staff)|govt\.? (?:officer|official)|officer|official|clerk|inspector|constable|head constable|sub-?inspector|tehsildar|patwari|talathi|revenue officer|municipal (?:officer|official|clerk)|peon|babu|customs officer|excise officer|income[- ]tax officer|registrar|sub-?registrar|engineer|doctor at the government hospital|teacher at the government school)).{0,90}(?:(?:asked for|asking for|ask for|demand|demands|demanded|demanding|took|take|takes|taking|accept|accepts|accepted|accepting|received|receiving|paid|pay|paying|gave|give|giving|offered|offering|collect|collects|collected|collecting)\s+(?:\w+\s+){0,3}?(?:bribe|money|cash|rs\.?\s*\d|rupees|₹\s*\d|commission|percentage|per cent|percent|cut|gift|gifts|speed money|under the table|hafta))|(?:(?:asked for|asking for|ask for|demand|demands|demanded|demanding|took|take|takes|taking|accept|accepts|accepted|accepting|received|receiving|paid|pay|paying|gave|give|giving|offered|offering|collect|collects|collected|collecting)\s+(?:\w+\s+){0,3}?(?:bribe|money|cash|rs\.?\s*\d|rupees|₹\s*\d|commission|percentage|per cent|percent|cut|gift|gifts|speed money|under the table|hafta)).{0,90}(?:(?:public servant|government (?:officer|official|servant|employee|staff)|govt\.? (?:officer|official)|officer|official|clerk|inspector|constable|head constable|sub-?inspector|tehsildar|patwari|talathi|revenue officer|municipal (?:officer|official|clerk)|peon|babu|customs officer|excise officer|income[- ]tax officer|registrar|sub-?registrar|engineer|doctor at the government hospital|teacher at the government school)))</t>
+          <t>(?:(?:(?:public servant|government (?:officer|official|servant|employee|staff)|govt\.? (?:officer|official)|officer|official|clerk|inspector|constable|head constable|sub-?inspector|tehsildar|patwari|talathi|revenue officer|municipal (?:officer|official|clerk)|peon|babu|customs officer|excise officer|income[- ]tax officer|registrar|sub-?registrar|engineer|doctor at the government hospital|teacher at the government school)).{0,90}(?:(?:asked (?:me |us |him |her )?for|asking (?:me |us |him |her )?for|ask for|demand|demands|demanded|demanding|took|take|takes|taking|accept|accepts|accepted|accepting|received|receiving|paid|pay|paying|gave|give|giving|offered|offering|collect|collects|collected|collecting)\s+(?:\w+\s+){0,3}?(?:bribe|money|cash|rs\.?\s*\d|rupees|₹\s*\d|commission|percentage|per cent|percent|cut|gift|gifts|speed money|under the table|hafta))|(?:(?:asked (?:me |us |him |her )?for|asking (?:me |us |him |her )?for|ask for|demand|demands|demanded|demanding|took|take|takes|taking|accept|accepts|accepted|accepting|received|receiving|paid|pay|paying|gave|give|giving|offered|offering|collect|collects|collected|collecting)\s+(?:\w+\s+){0,3}?(?:bribe|money|cash|rs\.?\s*\d|rupees|₹\s*\d|commission|percentage|per cent|percent|cut|gift|gifts|speed money|under the table|hafta)).{0,90}(?:(?:public servant|government (?:officer|official|servant|employee|staff)|govt\.? (?:officer|official)|officer|official|clerk|inspector|constable|head constable|sub-?inspector|tehsildar|patwari|talathi|revenue officer|municipal (?:officer|official|clerk)|peon|babu|customs officer|excise officer|income[- ]tax officer|registrar|sub-?registrar|engineer|doctor at the government hospital|teacher at the government school)))</t>
         </is>
       </c>
     </row>
@@ -1281,17 +1281,17 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>any use of terrorist / terrorism / terrorists / terrorise-type words (terroris + m or t ...)</t>
+          <t>'terrorist' / 'terrorism' / 'terrorists' within about 80 characters of a case word (booked, arrested, accused, charged, chargesheet, FIR, bail, case, trial, custody, detained, jail, police, court, NIA, 'under section' / 'under the')</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>The Act's own words (derived from its text)</t>
+          <t>Workbook, changed by me</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no (narrower than before; about the same as the workbook)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1301,12 +1301,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>From the Act's own vocabulary. LOOSER than the workbook, whose N2 needs 'terror...' NEAR booked / arrested / accused / charged / FIR / bail / case. A question that merely mentions terrorism fires it.</t>
+          <t>Workbook N2: terror... near booked / arrested / accused / charged / FIR / bail / case; I added a few more case words. CHANGED 2026-10-17 (weakness 3): it was a bare 'terroris-', which fired on any mention of terrorism, e.g. 'what is terrorism?'.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>\bterroris[mt]\w*</t>
+          <t>(?:(?:\bterroris[mt]\w*).{0,80}(?:\b(?:booked|arrest\w*|accused|charged?|charges|chargesheet|FIR|bail|case|cases|trial|custody|detained|detention|under (?:section|the)|jail|police|court|NIA)\b)|(?:\b(?:booked|arrest\w*|accused|charged?|charges|chargesheet|FIR|bail|case|cases|trial|custody|detained|detention|under (?:section|the)|jail|police|court|NIA)\b).{0,80}(?:\bterroris[mt]\w*))</t>
         </is>
       </c>
     </row>
@@ -1561,97 +1561,97 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>'banned' within 40 characters of organisation / outfit / group / association</t>
+          <t>'terrorist organisation(s)' / 'terrorist individual(s)' / 'terrorist list'</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Workbook, changed by me</t>
+          <t>The Act's own words (derived from its text)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>slightly</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 3 is 'banned organisation/group'; I added 'outfit' and 'association' and allowed other words in between.</t>
+          <t>The Act's own terms (schedule of terrorist organisations; designation of an individual as a terrorist). ADDED 2026-10-17 because tightening row 0 lost two of the 75 questions (UA04, UA06) that use them.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>(?:(?:\bbanned\b).{0,40}(?:\b(?:organi[sz]ation|outfit|group|association)\b)|(?:\b(?:organi[sz]ation|outfit|group|association)\b).{0,40}(?:\bbanned\b))</t>
+          <t>\bterrorist (?:organi[sz]ations?|individuals?|list)\b</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Prevention of Money-laundering Act, 2002 (PMLA)</t>
+          <t>Unlawful Activities (Prevention) Act, 1967 (UAPA)</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>'money laundering' / 'money-laundering' / 'laundered' / 'laundering'</t>
+          <t>declare / designate / notify / list (any form) within about 60 characters of 'terrorist' or 'terrorism'</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Workbook, changed by me</t>
+          <t>The Act's own words (derived from its text)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>slightly</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Workbook N1 anchor 2 is 'money laundering'; mine also catches laundered / laundering after it.</t>
+          <t>Mine, from the Act's s.35 (designating an organisation or an individual). ADDED 2026-10-17 for UA06 ('Can the Central Government declare an individual a terrorist ...').</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>\bmoney[- ]launder\w+</t>
+          <t>(?:(?:\b(?:declar\w+|designat\w+|notif\w+|list(?:ed)?)\b).{0,60}(?:\bterroris[mt]\w*)|(?:\bterroris[mt]\w*).{0,60}(?:\b(?:declar\w+|designat\w+|notif\w+|list(?:ed)?)\b))</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Prevention of Money-laundering Act, 2002 (PMLA)</t>
+          <t>Unlawful Activities (Prevention) Act, 1967 (UAPA)</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>'laundering' on its own</t>
+          <t>'banned' within 40 characters of organisation / outfit / group / association</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Mine (not in the workbook)</t>
+          <t>Workbook, changed by me</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>slightly</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1661,12 +1661,12 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Not in the workbook as a bare word.</t>
+          <t>Workbook N2 anchor 3 is 'banned organisation/group'; I added 'outfit' and 'association' and allowed other words in between.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>\blaundering\b</t>
+          <t>(?:(?:\bbanned\b).{0,40}(?:\b(?:organi[sz]ation|outfit|group|association)\b)|(?:\b(?:organi[sz]ation|outfit|group|association)\b).{0,40}(?:\bbanned\b))</t>
         </is>
       </c>
     </row>
@@ -1677,21 +1677,21 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>'proceeds of crime'</t>
+          <t>'money laundering' / 'money-laundering' / 'laundered' / 'laundering'</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Workbook, same words</t>
+          <t>Workbook, changed by me</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>slightly</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1701,12 +1701,12 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Workbook N1 anchor 3.</t>
+          <t>Workbook N1 anchor 2 is 'money laundering'; mine also catches laundered / laundering after it.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>\bproceeds of crime\b</t>
+          <t>\bmoney[- ]launder\w+</t>
         </is>
       </c>
     </row>
@@ -1717,21 +1717,21 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>'reporting entity' / 'reporting entities'</t>
+          <t>'laundering' on its own</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>The Act's own words (derived from its text)</t>
+          <t>Mine (not in the workbook)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1741,12 +1741,12 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Act's own vocabulary.</t>
+          <t>Not in the workbook as a bare word.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>\breporting entit\w+</t>
+          <t>\blaundering\b</t>
         </is>
       </c>
     </row>
@@ -1757,21 +1757,21 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>'adjudicating authority'</t>
+          <t>'proceeds of crime'</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>The Act's own words (derived from its text)</t>
+          <t>Workbook, same words</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1781,12 +1781,12 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Act's own vocabulary.</t>
+          <t>Workbook N1 anchor 3.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>\badjudicating authority\b</t>
+          <t>\bproceeds of crime\b</t>
         </is>
       </c>
     </row>
@@ -1797,21 +1797,21 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>'provisional attachment'</t>
+          <t>'reporting entity' / 'reporting entities'</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Workbook, changed by me</t>
+          <t>The Act's own words (derived from its text)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1821,12 +1821,12 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Workbook N1 needs 'PMLA', 'money laundering' or 'proceeds of crime' nearby; mine does not.</t>
+          <t>Act's own vocabulary.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>\bprovisional attachment\b</t>
+          <t>\breporting entit\w+</t>
         </is>
       </c>
     </row>
@@ -1837,21 +1837,21 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>'Enforcement Directorate' (spelled out)</t>
+          <t>'adjudicating authority'</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Workbook, same words</t>
+          <t>The Act's own words (derived from its text)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>same as workbook N2</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1861,12 +1861,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 2, bare. NOTE: the workbook's own False-Positive Audit says an agency name alone is not an Act marker ('ED acts under more than one regime'); N2 contradicts that and I followed N2. It is a judgement call; in practice almost every ED arrest is under the PMLA.</t>
+          <t>Act's own vocabulary.</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>\benforcement directorate\b</t>
+          <t>\badjudicating authority\b</t>
         </is>
       </c>
     </row>
@@ -1877,11 +1877,11 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>the capital letters ED (case-sensitive, so 'ed' inside a word never counts) within 60 characters of attach / froze / frozen / freeze / arrest / summon / raid / seize / notice / case / bail / questioned</t>
+          <t>'provisional attachment'</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>slightly</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1901,27 +1901,27 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 1; I added freez..., seiz... and questioned.</t>
+          <t>Workbook N1 needs 'PMLA', 'money laundering' or 'proceeds of crime' nearby; mine does not.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>(?:(?:(?-i:\bED\b)).{0,60}(?:\b(?:attach\w*|froze|frozen|freez\w*|arrest\w*|summon\w*|raid\w*|seiz\w*|notice|case|bail|questioned)\b)|(?:\b(?:attach\w*|froze|frozen|freez\w*|arrest\w*|summon\w*|raid\w*|seiz\w*|notice|case|bail|questioned)\b).{0,60}(?:(?-i:\bED\b)))</t>
+          <t>\bprovisional attachment\b</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Scheduled Castes and the Scheduled Tribes (Prevention of Atrocities) Act, 1989 (SC/ST Act)</t>
+          <t>Prevention of Money-laundering Act, 2002 (PMLA)</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>'caste name / caste abuse / caste slur / caste insult / caste-based / caste discrimination / caste remark'</t>
+          <t>'Enforcement Directorate' (spelled out) within about 80 characters of a cue: attach, froze/frozen/freeze, arrest, summon, raid, seize, notice, case, bail, questioned, ECIR, property, assets, bank, account, investigation, inquiry, enquiry, appear, laundering</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>slightly</t>
+          <t>no (narrower than before)</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -1941,37 +1941,37 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 1; 'caste remark' added.</t>
+          <t>Workbook N2 anchor 2 is the bare name. CHANGED 2026-10-17 (weakness 2): the workbook's own False-Positive Audit says an agency name alone is not an Act marker, so a cue word is now required (the same rule the 'ED' row already used). A question that only mentions the Directorate no longer fires.</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>\bcaste[- ](?:name|abuse|slur|insult|based|discrimination|remark)\b</t>
+          <t>(?:(?:\benforcement directorate\b).{0,80}(?:\b(?:attach\w*|froze|frozen|freez\w*|arrest\w*|summon\w*|raid\w*|seiz\w*|notice|case|bail|questioned|ECIR|propert\w+|assets?|bank|account|investigat\w*|inquir\w*|enquir\w*|appear\w*|launder\w*)\b)|(?:\b(?:attach\w*|froze|frozen|freez\w*|arrest\w*|summon\w*|raid\w*|seiz\w*|notice|case|bail|questioned|ECIR|propert\w+|assets?|bank|account|investigat\w*|inquir\w*|enquir\w*|appear\w*|launder\w*)\b).{0,80}(?:\benforcement directorate\b))</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Scheduled Castes and the Scheduled Tribes (Prevention of Atrocities) Act, 1989 (SC/ST Act)</t>
+          <t>Prevention of Money-laundering Act, 2002 (PMLA)</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>'because of my/his/her/their caste'</t>
+          <t>the capital letters ED (case-sensitive, so 'ed' inside a word never counts) within 60 characters of attach / froze / frozen / freeze / arrest / summon / raid / seize / notice / case / bail / questioned</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Workbook, same words</t>
+          <t>Workbook, changed by me</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>slightly</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1981,12 +1981,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 2.</t>
+          <t>Workbook N2 anchor 1; I added freez..., seiz... and questioned.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>\bbecause of (?:my|his|her|their) caste\b</t>
+          <t>(?:(?:(?-i:\bED\b)).{0,60}(?:\b(?:attach\w*|froze|frozen|freez\w*|arrest\w*|summon\w*|raid\w*|seiz\w*|notice|case|bail|questioned)\b)|(?:\b(?:attach\w*|froze|frozen|freez\w*|arrest\w*|summon\w*|raid\w*|seiz\w*|notice|case|bail|questioned)\b).{0,60}(?:(?-i:\bED\b)))</t>
         </is>
       </c>
     </row>
@@ -1997,21 +1997,21 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>'Dalit' or 'Adivasi'</t>
+          <t>'caste name / caste abuse / caste slur / caste insult / caste-based / caste discrimination / caste remark'</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Workbook, same words</t>
+          <t>Workbook, changed by me</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>slightly</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2021,12 +2021,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 3.</t>
+          <t>Workbook N2 anchor 1; 'caste remark' added.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>\b(?:dalit|adivasi)\b</t>
+          <t>\bcaste[- ](?:name|abuse|slur|insult|based|discrimination|remark)\b</t>
         </is>
       </c>
     </row>
@@ -2037,11 +2037,11 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>'Scheduled Caste(s)' / 'Scheduled Tribe(s)'</t>
+          <t>'because of my/his/her/their caste'</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2061,12 +2061,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 4 (also the Act's own words).</t>
+          <t>Workbook N2 anchor 2.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>\bscheduled (?:castes?|tribes?)\b</t>
+          <t>\bbecause of (?:my|his|her|their) caste\b</t>
         </is>
       </c>
     </row>
@@ -2077,21 +2077,21 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>'exclusive special court'</t>
+          <t>'Dalit' or 'Adivasi'</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>The Act's own words (derived from its text)</t>
+          <t>Workbook, same words</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2101,12 +2101,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Act's own vocabulary.</t>
+          <t>Workbook N2 anchor 3.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>\bexclusive special court\b</t>
+          <t>\b(?:dalit|adivasi)\b</t>
         </is>
       </c>
     </row>
@@ -2117,21 +2117,21 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>'atrocity / atrocities' within 100 characters of caste / tribe / tribal / Dalit / Adivasi / SC / ST</t>
+          <t>'Scheduled Caste(s)' / 'Scheduled Tribe(s)'</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Workbook, changed by me</t>
+          <t>Workbook, same words</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>slightly</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2141,37 +2141,37 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 5; I added Adivasi, SC and ST (SC/ST are matched in any case, so 'st' as a word can match).</t>
+          <t>Workbook N2 anchor 4 (also the Act's own words).</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>(?:(?:\batrocit(?:y|ies)\b).{0,100}(?:\b(?:caste|tribe|tribal|dalit|adivasi|sc|st)\b)|(?:\b(?:caste|tribe|tribal|dalit|adivasi|sc|st)\b).{0,100}(?:\batrocit(?:y|ies)\b))</t>
+          <t>\bscheduled (?:castes?|tribes?)\b</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Dowry Prohibition Act, 1961</t>
+          <t>Scheduled Castes and the Scheduled Tribes (Prevention of Atrocities) Act, 1989 (SC/ST Act)</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>'dowry' within 100 characters of demand... / given / giving / gave / taking / took / take / return... / agreement / articles</t>
+          <t>'exclusive special court'</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Workbook, changed by me</t>
+          <t>The Act's own words (derived from its text)</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>no (narrower than N2)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2181,37 +2181,37 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 is a bare 'dowry' (its own audit calls that too broad); workbook N1 has 'dowry' near demand / giving / taking / agreement. Mine is N1 plus given, gave, took, take, return..., articles. A 'dowry harassment under 498A' question does not fire unless it also has one of these words.</t>
+          <t>Act's own vocabulary.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>(?:(?:\bdowry\b).{0,100}(?:\b(?:demand\w*|given|giving|gave|taking|took|take|return\w*|agreement|articles)\b)|(?:\b(?:demand\w*|given|giving|gave|taking|took|take|return\w*|agreement|articles)\b).{0,100}(?:\bdowry\b))</t>
+          <t>\bexclusive special court\b</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Juvenile Justice (Care and Protection of Children) Act, 2015</t>
+          <t>Scheduled Castes and the Scheduled Tribes (Prevention of Atrocities) Act, 1989 (SC/ST Act)</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>'juvenile'</t>
+          <t>'atrocity / atrocities' within 100 characters of caste / tribe / tribal / Dalit / Adivasi / SC / ST</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Workbook, same words</t>
+          <t>Workbook, changed by me</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>slightly</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2221,37 +2221,37 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 1.</t>
+          <t>Workbook N2 anchor 5; I added Adivasi, SC and ST (SC/ST are matched in any case, so 'st' as a word can match).</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>\bjuvenile\b</t>
+          <t>(?:(?:\batrocit(?:y|ies)\b).{0,100}(?:\b(?:caste|tribe|tribal|dalit|adivasi|sc|st)\b)|(?:\b(?:caste|tribe|tribal|dalit|adivasi|sc|st)\b).{0,100}(?:\batrocit(?:y|ies)\b))</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Juvenile Justice (Care and Protection of Children) Act, 2015</t>
+          <t>Dowry Prohibition Act, 1961</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>'juvenile justice board'</t>
+          <t>'dowry' within 100 characters of demand... / given / giving / gave / taking / took / take / return... / agreement / articles</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Workbook, same words</t>
+          <t>Workbook, changed by me</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>no (narrower than N2)</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2261,12 +2261,12 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Workbook N1 anchor 2.</t>
+          <t>Workbook N2 is a bare 'dowry' (its own audit calls that too broad); workbook N1 has 'dowry' near demand / giving / taking / agreement. Mine is N1 plus given, gave, took, take, return..., articles. A 'dowry harassment under 498A' question does not fire unless it also has one of these words.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>\bjuvenile justice board\b</t>
+          <t>(?:(?:\bdowry\b).{0,100}(?:\b(?:demand\w*|given|giving|gave|taking|took|take|return\w*|agreement|articles)\b)|(?:\b(?:demand\w*|given|giving|gave|taking|took|take|return\w*|agreement|articles)\b).{0,100}(?:\bdowry\b))</t>
         </is>
       </c>
     </row>
@@ -2277,11 +2277,11 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>'child in conflict with law'</t>
+          <t>'juvenile'</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2301,12 +2301,12 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Workbook N1 anchor 3.</t>
+          <t>Workbook N2 anchor 1.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>\bchild in conflict with law\b</t>
+          <t>\bjuvenile\b</t>
         </is>
       </c>
     </row>
@@ -2317,11 +2317,11 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>'child in need of care and protection'</t>
+          <t>'juvenile justice board'</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -2341,12 +2341,12 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Workbook N1 anchor 4.</t>
+          <t>Workbook N1 anchor 2.</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>\bchild in need of care and protection\b</t>
+          <t>\bjuvenile justice board\b</t>
         </is>
       </c>
     </row>
@@ -2357,11 +2357,11 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>'observation home'</t>
+          <t>'child in conflict with law'</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2381,12 +2381,12 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 4.</t>
+          <t>Workbook N1 anchor 3.</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>\bobservation home\b</t>
+          <t>\bchild in conflict with law\b</t>
         </is>
       </c>
     </row>
@@ -2397,21 +2397,21 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>'child welfare committee'</t>
+          <t>'child in need of care and protection'</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Workbook map, used by me as a question trigger</t>
+          <t>Workbook, same words</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2421,12 +2421,12 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>In Mr. Advocate's map as a passage marker, not in Machine Spec v2's question anchors.</t>
+          <t>Workbook N1 anchor 4.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>\bchild welfare committee\b</t>
+          <t>\bchild in need of care and protection\b</t>
         </is>
       </c>
     </row>
@@ -2437,21 +2437,21 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>'proof of age' / 'age determination' / 'age of the child/accused' within 100 characters of child / minor / school certificate / Aadhaar / birth certificate</t>
+          <t>'observation home'</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Workbook, changed by me</t>
+          <t>Workbook, same words</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>no (narrower)</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2461,12 +2461,12 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 5 is a bare 'proof of age|age determination'; mine needs a child word nearby (narrower).</t>
+          <t>Workbook N2 anchor 4.</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>(?:(?:\b(?:proof of age|age determination|age of the (?:child|accused))\b).{0,100}(?:\b(?:child|minor|school certificate|aadhaar|birth certificate)\b)|(?:\b(?:child|minor|school certificate|aadhaar|birth certificate)\b).{0,100}(?:\b(?:proof of age|age determination|age of the (?:child|accused))\b))</t>
+          <t>\bobservation home\b</t>
         </is>
       </c>
     </row>
@@ -2477,21 +2477,21 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>'minor' or a 5-17 year old within 60 characters of arrest / accused / custody / jail / remand / police station</t>
+          <t>'child welfare committee'</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Workbook, changed by me</t>
+          <t>Workbook map, used by me as a question trigger</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>slightly</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2501,27 +2501,27 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchors 2 and 3 merged; I added remand and police station and dropped 'theft' and 'fight'.</t>
+          <t>In Mr. Advocate's map as a passage marker, not in Machine Spec v2's question anchors.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>(?:(?:\b(?:minor|(?:1[0-7]|[5-9])[- ]?year[- ]?old)\b).{0,60}(?:\b(?:arrest\w*|accused|custody|jail|remand|police station)\b)|(?:\b(?:arrest\w*|accused|custody|jail|remand|police station)\b).{0,60}(?:\b(?:minor|(?:1[0-7]|[5-9])[- ]?year[- ]?old)\b))</t>
+          <t>\bchild welfare committee\b</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Arms Act, 1959</t>
+          <t>Juvenile Justice (Care and Protection of Children) Act, 2015</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>gun / pistol / revolver / rifle / firearm / bullet(s) / cartridge(s) / ammunition within 80 characters of found / recovered / seized / caught / carrying / carried / licence / unlicensed / possession / police</t>
+          <t>'proof of age' / 'age determination' / 'age of the child/accused' within 100 characters of child / minor / school certificate / Aadhaar / birth certificate</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>slightly</t>
+          <t>no (narrower)</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2541,37 +2541,37 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 1; I added ammunition, carried, licence, unlicensed, possession and dropped 'car', 'bag', 'without'.</t>
+          <t>Workbook N2 anchor 5 is a bare 'proof of age|age determination'; mine needs a child word nearby (narrower).</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>(?:(?:\b(?:gun|pistol|revolver|rifle|firearm|bullets?|cartridges?|ammunition)\b).{0,80}(?:\b(?:found|recovered|seized|caught|carrying|carried|licen[cs]e|unlicensed|possession|police)\b)|(?:\b(?:found|recovered|seized|caught|carrying|carried|licen[cs]e|unlicensed|possession|police)\b).{0,80}(?:\b(?:gun|pistol|revolver|rifle|firearm|bullets?|cartridges?|ammunition)\b))</t>
+          <t>(?:(?:\b(?:proof of age|age determination|age of the (?:child|accused))\b).{0,100}(?:\b(?:child|minor|school certificate|aadhaar|birth certificate)\b)|(?:\b(?:child|minor|school certificate|aadhaar|birth certificate)\b).{0,100}(?:\b(?:proof of age|age determination|age of the (?:child|accused))\b))</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Motor Vehicles Act, 1988</t>
+          <t>Juvenile Justice (Care and Protection of Children) Act, 2015</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>'drunk driving' / 'drunken driving'</t>
+          <t>'minor' or a 5-17 year old within 60 characters of arrest / accused / custody / jail / remand / police station</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Workbook, same words</t>
+          <t>Workbook, changed by me</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>slightly</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2581,27 +2581,27 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Workbook N1 anchor 2.</t>
+          <t>Workbook N2 anchors 2 and 3 merged; I added remand and police station and dropped 'theft' and 'fight'.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>\bdrunk(?:en)? driving\b</t>
+          <t>(?:(?:\b(?:minor|(?:1[0-7]|[5-9])[- ]?year[- ]?old)\b).{0,60}(?:\b(?:arrest\w*|accused|custody|jail|remand|police station)\b)|(?:\b(?:arrest\w*|accused|custody|jail|remand|police station)\b).{0,60}(?:\b(?:minor|(?:1[0-7]|[5-9])[- ]?year[- ]?old)\b))</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Motor Vehicles Act, 1988</t>
+          <t>Arms Act, 1959</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>'drink and drive' / 'drink-and-driving'</t>
+          <t>gun / pistol / revolver / rifle / firearm / bullet(s) / cartridge(s) / ammunition within 80 characters of found / recovered / seized / caught / carrying / carried / licence / unlicensed / possession / police</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2621,12 +2621,12 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 5 is 'drunk and driv...'; mine is 'drink and driv...'.</t>
+          <t>Workbook N2 anchor 1; I added ammunition, carried, licence, unlicensed, possession and dropped 'car', 'bag', 'without'.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>\bdrink[- ]and[- ]driv\w+</t>
+          <t>(?:(?:\b(?:gun|pistol|revolver|rifle|firearm|bullets?|cartridges?|ammunition)\b).{0,80}(?:\b(?:found|recovered|seized|caught|carrying|carried|licen[cs]e|unlicensed|possession|police)\b)|(?:\b(?:found|recovered|seized|caught|carrying|carried|licen[cs]e|unlicensed|possession|police)\b).{0,80}(?:\b(?:gun|pistol|revolver|rifle|firearm|bullets?|cartridges?|ammunition)\b))</t>
         </is>
       </c>
     </row>
@@ -2637,11 +2637,11 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>'hit and run'</t>
+          <t>'drunk driving' / 'drunken driving'</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2661,12 +2661,12 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 2.</t>
+          <t>Workbook N1 anchor 2.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>\bhit[- ]and[- ]run\b</t>
+          <t>\bdrunk(?:en)? driving\b</t>
         </is>
       </c>
     </row>
@@ -2677,21 +2677,21 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>'dangerous driving'</t>
+          <t>'drink and drive' / 'drink-and-driving'</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Workbook, same words</t>
+          <t>Workbook, changed by me</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>slightly</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2701,12 +2701,12 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 anchor 4.</t>
+          <t>Workbook N2 anchor 5 is 'drunk and driv...'; mine is 'drink and driv...'.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>\bdangerous driving\b</t>
+          <t>\bdrink[- ]and[- ]driv\w+</t>
         </is>
       </c>
     </row>
@@ -2717,34 +2717,114 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>'hit and run'</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Workbook, same words</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Workbook N2 anchor 2.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>\bhit[- ]and[- ]run\b</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Motor Vehicles Act, 1988</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>'dangerous driving'</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Workbook, same words</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Workbook N2 anchor 4.</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>\bdangerous driving\b</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Motor Vehicles Act, 1988</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>'driving without a (valid) licence / insurance', 'driving under the influence', 'driving after drinking'</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>Workbook, changed by me</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>slightly</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>Workbook N1 anchor 3 and N2 anchors 3 and 6, merged; 'insurance' is mine.</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>\bdriving (?:without (?:a )?(?:valid )?(?:licen[cs]e|insurance)|under the influence|after drinking)\b</t>
         </is>
@@ -2805,12 +2885,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>The word pass for this Act does NOT fire at all if the question contains any of: private company / firm / sector / bank / hospital / school / college, my boss, shopkeeper, landlord, builder, 'contractor asked me', voter(s), election(s), poll, polling, candidate.</t>
+          <t>Two guards. (1) The word pass for this Act does NOT fire at all if the question contains voter(s), election(s), poll, polling or candidate (election bribery is a different offence). (2) It does NOT fire if the question contains private company / firm / sector / bank / hospital / school / college, my boss, shopkeeper, landlord, builder or 'contractor asked me' -- UNLESS the question also names a public servant (public servant, government/govt officer / official / clerk / hospital / school ..., sarkari, police / policeman, constable, inspector, sub-inspector, tehsildar, patwari, talathi, revenue officer, municipal, panchayat, customs / excise / income-tax officer, registrar, babu, vigilance, anti-corruption).</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>The PRINCIPLE is the workbook's (layperson sheet: a private-sector payment is not automatically a Prevention of Corruption Act matter; Mr. Advocate's map: election bribery is a different offence). The WORD LIST is mine. WEAKNESS: it is blunt. 'I am a builder and the municipal officer asked me for Rs 50,000 to approve my plan' contains 'builder' and is therefore NOT matched, although a public servant is plainly involved.</t>
+          <t>The PRINCIPLE is the workbook's (layperson sheet: a private-sector payment is not automatically a Prevention of Corruption Act matter; Mr. Advocate's map: election bribery is a different offence). The WORD LIST is mine. CHANGED 2026-10-17 (weakness 1): guard (2) used to be absolute, so 'I am a builder and the municipal officer asked me for Rs 50,000' was not matched. The 'public servant' list for lifting it is stricter than the role list in row 9, because a bare 'officer' or 'clerk' can work in a private firm. Election words still block even with a public servant named.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs, sheet and patch copies for the four added Directory Acts (34 rows)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YEUNXbYb9LDbJLc2ziqL3n
</commit_message>
<xml_diff>
--- a/acts/ACT_TRIGGER_LIST.xlsx
+++ b/acts/ACT_TRIGGER_LIST.xlsx
@@ -2949,7 +2949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4536,6 +4536,222 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Prohibition of Child Marriage Act, 2006</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>child_marriage_act_2006</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>names / aliases ('This question NAMES the ...')</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>prohibition of child marriage act; child marriage act; pcma; child marriage prohibition act</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Directory, written 2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Prohibition of Child Marriage Act, 2006</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>child_marriage_act_2006</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>phrases ('looks like it is about the ...')</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>child marriage; child marriages; underage marriage; underage marriages; underage wedding; child marriage prohibition officer; married below the legal age; marriage below the legal age</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Directory, written 2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Protection of Civil Rights Act, 1955</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>pcr_act_1955</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>names / aliases ('This question NAMES the ...')</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>protection of civil rights act; pcr act; untouchability offences act; civil rights act 1955</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Directory, written 2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Protection of Civil Rights Act, 1955</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>pcr_act_1955</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>phrases ('looks like it is about the ...')</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>practice of untouchability; practising untouchability; practicing untouchability; enforcing untouchability; untouchability offence; untouchability offences; untouchability case</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Directory, written 2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Prevention of Damage to Public Property Act, 1984</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>pdpp_act_1984</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>names / aliases ('This question NAMES the ...')</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>prevention of damage to public property act; damage to public property act; pdpp act; pdpp</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Directory, written 2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Prevention of Damage to Public Property Act, 1984</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>pdpp_act_1984</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>phrases ('looks like it is about the ...')</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>damage to public property; damaging public property; damaged public property; destruction of public property; destroying public property; destroyed public property; public property damage</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Directory, written 2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>muslim_women_act_2019</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>names / aliases ('This question NAMES the ...')</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>muslim women protection of rights on marriage act; muslim women act 2019; triple talaq act; triple talaq law</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Directory, written 2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>muslim_women_act_2019</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>phrases ('looks like it is about the ...')</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>triple talaq; instant talaq; talaq e biddat; pronounced talaq three times; talaq three times</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Directory, written 2026-10-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4547,7 +4763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -5045,6 +5261,74 @@
       <c r="C29" s="2" t="inlineStr">
         <is>
           <t>the time limit for bringing a case to court, and when a delay can be condoned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Prohibition of Child Marriage Act, 2006</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>child_marriage_act_2006</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>a child marriage (a girl under 18 or a boy under 21 married): making it voidable, stopping it by court injunction, and the punishment of those who arrange or conduct it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Protection of Civil Rights Act, 1955</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>pcr_act_1955</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>the practice of untouchability: refusing a person entry to a temple, well, shop, hospital or public place, or other social disabilities, because of 'untouchability' (a different Act from the SC/ST Atrocities Act).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Prevention of Damage to Public Property Act, 1984</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>pdpp_act_1984</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>damage to public property: a bus, train, government building or other public property damaged or burned in a protest, riot or bandh, and the special bail rule for it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>muslim_women_act_2019</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>instant triple talaq (talaq-e-biddat): pronouncing talaq three times at once, which the Act makes void and punishable, with the wife's subsistence allowance and custody of her minor children.</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5430,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>No word pass. ITPA, CGST and the Companies Act are in the Directory (names/phrases) and can be chosen by the AI pass; the Child Marriage, Civil Rights, Public Property and Muslim Women Acts are not in the Directory at all yet.</t>
+          <t>No word pass. All seven are in the Directory (names/phrases) and can be chosen by the AI pass. The Child Marriage, Civil Rights, Public Property and Muslim Women Acts were added to the Directory on 2026-10-17 with names and phrases drawn from the workbook's own strong terms; their false-positive notes (child marriage also arises under POCSO and personal law; the PCR Act is not the SC/ST Act; triple talaq also arises in constitutional discussion) are why they get no word pass.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs, evidence files, trigger list and patch copies for the Muslim Women and Public Property word passes (FOLLOW_UPS 2at, DEPLOY_STAGING Part 4n)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YEUNXbYb9LDbJLc2ziqL3n
</commit_message>
<xml_diff>
--- a/acts/ACT_TRIGGER_LIST.xlsx
+++ b/acts/ACT_TRIGGER_LIST.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Everyday wording and the Acts' own vocabulary, by regular expression, for nine Acts (sheet 'Layer 2'). Built in four steps: (1) I started from the owner's trigger workbook, Machine Spec v2 (N1 precise anchors, N2 plain-language anchors, and the exclusion guards), which Mr. Advocate's regex audit had repaired; (2) I tested the layperson sheet's own phrases as matchers and rejected them (3-12%); (3) I derived each loaded Act's distinctive vocabulary by program (words the Act uses that the BNS/BNSS and the other four Acts rarely do) and pruned it by hand; (4) I rewrote every pattern BY HAND into the code (nothing was pasted as it is), changing or adding to it as the 'Source' column says. Some changes were made AFTER I had seen which of my 75 test questions were missed or after the owner's staging sentences: those rows say so, and they make the 84% score an optimistic ceiling.</t>
+          <t>Everyday wording and the Acts' own vocabulary, by regular expression, for eleven Acts (sheet 'Layer 2'). Built in four steps: (1) I started from the owner's trigger workbook, Machine Spec v2 (N1 precise anchors, N2 plain-language anchors, and the exclusion guards), which Mr. Advocate's regex audit had repaired; (2) I tested the layperson sheet's own phrases as matchers and rejected them (3-12%); (3) I derived each loaded Act's distinctive vocabulary by program (words the Act uses that the BNS/BNSS and the other four Acts rarely do) and pruned it by hand; (4) I rewrote every pattern BY HAND into the code (nothing was pasted as it is), changing or adding to it as the 'Source' column says. The Muslim Women and Public Property Acts (added 2026-10-17) were tested on 64 questions frozen BEFORE their patterns were written (first run: 16/16, 18/18, no false alarm in 30 near-misses) and then on 60 harder ones (first run: 14/16, 13/17, 3 false alarms in 27), after which the patterns were tightened (rows marked 'yes' in the 'after misses' column). Some changes were made AFTER I had seen which of my 75 test questions were missed or after the owner's staging sentences: those rows say so, and they make the 84% score an optimistic ceiling.</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2830,6 +2830,806 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>'teen talaq', 'three talaq' or '3 talaq' (also 'teen baar talaq', 'three times talaq'; spellings talaq / talaaq / talak / thalaq)</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>From the Layperson Trigger Additions ('husband said talaq three times at once', 'teen talaq'). The Directory holds only the exact phrase 'triple talaq'.</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>\b(?:teen|three|3)\s+(?:baar\s+|times\s+)?th?ala{1,2}[qk]s?\b</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>the word talaq three times in a row ('talaq, talaq, talaq'), with at most two words between</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Same sheet ('husband pronounced talaq three times').</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>\bth?ala{1,2}[qk]\w*\W+(?:\w+\W+){0,2}?\bth?ala{1,2}[qk]\w*\W+(?:\w+\W+){0,2}?\bth?ala{1,2}[qk]\w*</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>talaq within 40 characters of 'three times', 'thrice' or 'teen baar'</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Same sheet.</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:\bth?ala{1,2}[qk]\w*).{0,40}(?:(?:\b(?:three|3)\s+times\b|\bthrice\b|\b(?:teen|tin)\s+baar\b))|(?:(?:\b(?:three|3)\s+times\b|\bthrice\b|\b(?:teen|tin)\s+baar\b)).{0,40}(?:\bth?ala{1,2}[qk]\w*))</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>'triple talaq' in other spellings (triple talak, tripple talaaq ...)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>The Directory's phrase 'triple talaq' needs the exact spelling.</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>\btrip{1,2}le\s+th?ala{1,2}[qk]\b</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>talaq-e-biddat and its spellings (talaq e bidat, talaq-ul-biddat, talaq i biddat ...)</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>The Revised Trigger Map names talaq-e-biddat as the STRONG term. The Directory holds the exact 'talaq e biddat'.</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>\bth?ala{1,2}[qk]\W{0,3}(?:(?:e|i|ul)\W{0,3})?bi?dd?at\b</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>talaq within 60 characters of: instant, immediate(ly), irrevocable, at once, in one go, in one sitting, in a single breath, in one sentence, on the spot</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Layperson sheet ('instant talaq message', 'instant divorce announcement'). 'In a single breath / one sentence' was added after the harder question set missed 'oral talaq in anger in a single breath'.</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:\bth?ala{1,2}[qk]\w*).{0,60}(?:(?:\binstant\w*|\bimmediate\w*|\birrevocabl\w+|\bat\s+once\b|\bin\s+(?:a\s+)?(?:one|single)\s+(?:go|sitting|breath|stroke|sentence)\b|\b(?:one|single)\s+sitting\b|\bon\s+the\s+spot\b))|(?:(?:\binstant\w*|\bimmediate\w*|\birrevocabl\w+|\bat\s+once\b|\bin\s+(?:a\s+)?(?:one|single)\s+(?:go|sitting|breath|stroke|sentence)\b|\b(?:one|single)\s+sitting\b|\bon\s+the\s+spot\b)).{0,60}(?:\bth?ala{1,2}[qk]\w*))</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>talaq within 50 characters of: WhatsApp, SMS, text (message), email, letter, speed post, registered post, courier, stamp paper, voice message, voicemail, video call, Instagram, Facebook, Telegram, messenger, 'over the phone', 'phone call'</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Layperson sheet ('triple talaq over phone or WhatsApp'). A bare 'phone' or 'message' was REMOVED after the harder question set: 'he said he will give me talaq if I speak to my parents on the phone' is a threat, not a pronouncement. Instagram, Facebook, Telegram and the phone-call forms were added in the same pass.</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:\bth?ala{1,2}[qk]\w*).{0,50}(?:(?:\bwhatsapp\b|\bsms\b|\btext(?:\s+message)?\b|\be-?mail\b|\bletter\b|\bspeed\s+post\b|\bregistered\s+post\b|\bcourier\b|\bstamp\s+paper\b|\bvoice\s+(?:message|note)\b|\bvoicemail\b|\bvideo\s+call\b|\binstagram\b|\bfacebook\b|\btelegram\b|\bmessenger\b|\bover\s+(?:the\s+)?(?:phone|telephone)\b|\bphone\s+call\b))|(?:(?:\bwhatsapp\b|\bsms\b|\btext(?:\s+message)?\b|\be-?mail\b|\bletter\b|\bspeed\s+post\b|\bregistered\s+post\b|\bcourier\b|\bstamp\s+paper\b|\bvoice\s+(?:message|note)\b|\bvoicemail\b|\bvideo\s+call\b|\binstagram\b|\bfacebook\b|\btelegram\b|\bmessenger\b|\bover\s+(?:the\s+)?(?:phone|telephone)\b|\bphone\s+call\b)).{0,50}(?:\bth?ala{1,2}[qk]\w*))</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>talaq within 60 characters of: FIR, police, arrest, jail, bail, imprisonment, criminal, punish(ment), offence, three years, cognizable, compoundable</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>The Act makes the pronouncement a criminal offence (section 4, cognizable and non-bailable-style bail rules in section 7); the workbook's note says to use it where 'a criminal/enforcement context' is present.</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:\bth?ala{1,2}[qk]\w*).{0,60}(?:(?:\bFIR\b|\bpolice\b|\barrest\w*|\bjail\b|\bbail\b|\bimprison\w*|\bcriminal\b|\bpunish\w*|\boffence\b|\bthree\s+years\b|\bcognizable\b|\bcompoundable\b))|(?:(?:\bFIR\b|\bpolice\b|\barrest\w*|\bjail\b|\bbail\b|\bimprison\w*|\bcriminal\b|\bpunish\w*|\boffence\b|\bthree\s+years\b|\bcognizable\b|\bcompoundable\b)).{0,60}(?:\bth?ala{1,2}[qk]\w*))</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>talaq within 100 characters of 'subsistence allowance'</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>The Act's own term (section 5).</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:\bth?ala{1,2}[qk]\w*).{0,100}(?:\bsubsistence\s+allowance\b)|(?:\bsubsistence\s+allowance\b).{0,100}(?:\bth?ala{1,2}[qk]\w*))</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>'Muslim Women Act' (with or without a bracketed title) within 80 characters of talaq, 'triple' or '2019'</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>The bare name 'Muslim Women Act' is NOT in the Directory because the Muslim Women (Protection of Rights on Divorce) Act, 1986 is a different Act; the added word keeps the two apart.</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:\bmuslim\s+women(?:'s)?\s+(?:\([^)]{0,40}\)\s*)?act\b).{0,80}(?:\bth?ala{1,2}[qk]\w*|\btriple\b|\b2019\b)|(?:\bth?ala{1,2}[qk]\w*|\btriple\b|\b2019\b).{0,80}(?:\bmuslim\s+women(?:'s)?\s+(?:\([^)]{0,40}\)\s*)?act\b))</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>'divorce' (any form) within 70 characters of a delivery or instant word (WhatsApp, SMS, text message, email, letter, speed post, stamp paper, voice message, video call, thrice, instant, immediate, at once, in one go, on the spot), AND the question says Muslim / Islamic / shariat / nikah / qazi within 250 characters</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>For a question that never uses the word talaq ('a Muslim husband divorced her by email'). The religion word is required because the same facts under another personal law are not this Act. 'Thrice' and 'qazi' were added after the harder question set.</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:(?:(?:\bdivorc\w+).{0,70}(?:(?:\bwhatsapp\b|\bsms\b|\btext\s+message\b|\be-?mail\b|\bletter\b|\bspeed\s+post\b|\bstamp\s+paper\b|\bvoice\s+(?:message|note)\b|\bvideo\s+call\b|\bthrice\b|(?:\binstant\w*|\bimmediate\w*|\birrevocabl\w+|\bat\s+once\b|\bin\s+(?:a\s+)?(?:one|single)\s+(?:go|sitting|breath|stroke|sentence)\b|\b(?:one|single)\s+sitting\b|\bon\s+the\s+spot\b)))|(?:(?:\bwhatsapp\b|\bsms\b|\btext\s+message\b|\be-?mail\b|\bletter\b|\bspeed\s+post\b|\bstamp\s+paper\b|\bvoice\s+(?:message|note)\b|\bvideo\s+call\b|\bthrice\b|(?:\binstant\w*|\bimmediate\w*|\birrevocabl\w+|\bat\s+once\b|\bin\s+(?:a\s+)?(?:one|single)\s+(?:go|sitting|breath|stroke|sentence)\b|\b(?:one|single)\s+sitting\b|\bon\s+the\s+spot\b))).{0,70}(?:\bdivorc\w+))).{0,250}(?:\b(?:muslim|islam\w*|shariat|sharia\w*|shariah|nikah\w*|qazi)\b)|(?:\b(?:muslim|islam\w*|shariat|sharia\w*|shariah|nikah\w*|qazi)\b).{0,250}(?:(?:(?:\bdivorc\w+).{0,70}(?:(?:\bwhatsapp\b|\bsms\b|\btext\s+message\b|\be-?mail\b|\bletter\b|\bspeed\s+post\b|\bstamp\s+paper\b|\bvoice\s+(?:message|note)\b|\bvideo\s+call\b|\bthrice\b|(?:\binstant\w*|\bimmediate\w*|\birrevocabl\w+|\bat\s+once\b|\bin\s+(?:a\s+)?(?:one|single)\s+(?:go|sitting|breath|stroke|sentence)\b|\b(?:one|single)\s+sitting\b|\bon\s+the\s+spot\b)))|(?:(?:\bwhatsapp\b|\bsms\b|\btext\s+message\b|\be-?mail\b|\bletter\b|\bspeed\s+post\b|\bstamp\s+paper\b|\bvoice\s+(?:message|note)\b|\bvideo\s+call\b|\bthrice\b|(?:\binstant\w*|\bimmediate\w*|\birrevocabl\w+|\bat\s+once\b|\bin\s+(?:a\s+)?(?:one|single)\s+(?:go|sitting|breath|stroke|sentence)\b|\b(?:one|single)\s+sitting\b|\bon\s+the\s+spot\b))).{0,70}(?:\bdivorc\w+))))</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>'I divorce you' / 'divorced me' said three times, AND the question says Muslim / Islamic / shariat / nikah / qazi</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>'Three times' alone near 'divorce' fires on 'I called her three times', so the pattern needs 'divorce you / divorced me ... three times' as one phrase.</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:\bdivorce\s+(?:you|her)\b.{0,30}\b(?:three|3)\s+times\b|\b(?:three|3)\s+times\b.{0,30}\bdivorce\s+you\b|\bdivorc\w+\s+(?:me|her)\s+(?:by\s+saying\s+\S+\s+)?(?:\w+\s+){0,3}(?:three|3)\s+times\b).{0,250}(?:\b(?:muslim|islam\w*|shariat|sharia\w*|shariah|nikah\w*|qazi)\b)|(?:\b(?:muslim|islam\w*|shariat|sharia\w*|shariah|nikah\w*|qazi)\b).{0,250}(?:\bdivorce\s+(?:you|her)\b.{0,30}\b(?:three|3)\s+times\b|\b(?:three|3)\s+times\b.{0,30}\bdivorce\s+you\b|\bdivorc\w+\s+(?:me|her)\s+(?:by\s+saying\s+\S+\s+)?(?:\w+\s+){0,3}(?:three|3)\s+times\b))</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Prevention of Damage to Public Property Act, 1984</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>a damage word (damage, destroy, burn, torch, set fire, arson, vandalise, smash, ransack, stone, throw stones, break) next to 'public / government / state / railway / municipal / panchayat property', as the verb's object (within 3 words) or as 'the property was ...'</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>From the Revised Trigger Map ('damage to public property during protest/riot'). Needs the noun 'property' with a public word, so 'broke his promise to the government' never fires.</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:(?:(?:\bset(?:ting|s)?\s+fire\b|\btorch\w*|\barson\w*|\bburn\w*|\bgutted\b|\bvandali[sz]\w*|\bransack\w*|\bsmash\w*|\bstoned\b|\bstone[- ]?pelt\w*|\bset(?:ting|s)?\s+ablaze\b|\b(?:threw|thrown|throwing|throw|throws|pelt\w*|hurl\w*)\s+(?:\w+\s+){0,2}?(?:stones?|bricks?|petrol\s+bombs?|bottles?)\b|\bpetrol\s+bombs?\b)|\b(?:break(?:ing|s)?|broke|broken)\s+(?:\w+\s+){0,3}?(?:windows?|windscreens?|windshields?|glass|doors?|gates?|furniture|signals?|lights?|barricades?)\b|(?:\bdamag\w+|\bdestr(?:oy\w*|uction|uctive)\b|\bwreck\w*|\bruin\w*))|\b(?:break(?:ing|s)?|broke|broken)\b)\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,3}?\b(?:public|government|govt\.?|state|railway|railways|municipal|panchayat)\s+propert(?:y|ies)\b|\b(?:public|government|govt\.?|state|railway|railways|municipal|panchayat)\s+propert(?:y|ies)\b\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,3}?(?:was|were|got|gets|is|are|been|being)\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,2}?(?:(?:(?:\bset(?:ting|s)?\s+fire\b|\btorch\w*|\barson\w*|\bburn\w*|\bgutted\b|\bvandali[sz]\w*|\bransack\w*|\bsmash\w*|\bstoned\b|\bstone[- ]?pelt\w*|\bset(?:ting|s)?\s+ablaze\b|\b(?:threw|thrown|throwing|throw|throws|pelt\w*|hurl\w*)\s+(?:\w+\s+){0,2}?(?:stones?|bricks?|petrol\s+bombs?|bottles?)\b|\bpetrol\s+bombs?\b)|\b(?:break(?:ing|s)?|broke|broken)\s+(?:\w+\s+){0,3}?(?:windows?|windscreens?|windshields?|glass|doors?|gates?|furniture|signals?|lights?|barricades?)\b|(?:\bdamag\w+|\bdestr(?:oy\w*|uction|uctive)\b|\bwreck\w*|\bruin\w*))|\b(?:break(?:ing|s)?|broke|broken)\b))</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Prevention of Damage to Public Property Act, 1984</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>'public property damage', 'government property destruction' (property noun, then damage / destruction / vandalism / arson)</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Same.</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>\b(?:public|government|govt\.?|state|railway|railways|municipal|panchayat)\s+propert(?:y|ies)\b\s+(?:damage|destruction|vandalism|arson)\b</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Prevention of Damage to Public Property Act, 1984</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>a violent verb (burn, torch, set fire, arson, vandalise, smash, ransack, stone, throw stones / bricks / petrol bombs, break the windows / glass / doors / gates of ...) with a public thing as its OBJECT within 5 words, or 'the bus was burnt'. Public things: public or government or state bus / building / office / school / hospital / vehicle, state transport or roadways bus, RTC / DTC bus, railway station / track / coach / engine / signal, police station / vehicle / jeep, municipal or panchayat or tehsil office, collectorate, post office, court building, bus stand or depot, metro train or station, toll plaza, street / signal / traffic lights. No protest word is needed.</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Layperson sheet ('public office set on fire', 'railway or public transport property vandalised'). Rewritten after the harder question set: the thing must be the OBJECT of the verb, so 'someone smashed my phone and I went to the police station' no longer counts. Words that mean the person went and reported something are not allowed inside the stretch.</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:(?:\bset(?:ting|s)?\s+fire\b|\btorch\w*|\barson\w*|\bburn\w*|\bgutted\b|\bvandali[sz]\w*|\bransack\w*|\bsmash\w*|\bstoned\b|\bstone[- ]?pelt\w*|\bset(?:ting|s)?\s+ablaze\b|\b(?:threw|thrown|throwing|throw|throws|pelt\w*|hurl\w*)\s+(?:\w+\s+){0,2}?(?:stones?|bricks?|petrol\s+bombs?|bottles?)\b|\bpetrol\s+bombs?\b)|\b(?:break(?:ing|s)?|broke|broken)\s+(?:\w+\s+){0,3}?(?:windows?|windscreens?|windshields?|glass|doors?|gates?|furniture|signals?|lights?|barricades?)\b)\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,5}?(?:\bpublic\s+(?:building|buildings|transport|vehicle|vehicles|bus|buses|utility|utilities|asset|assets|toilets?|library|park)\b|\b(?:government|govt\.?|state)\s+(?:building|buildings|office|offices|vehicle|vehicles|bus|buses|school|schools|hospital|hospitals|college|colleges|premises|asset|assets|establishment|establishments|transport|jeeps?|guest\s+house)\b|\b(?:state\s+transport|roadways|road\s+transport)\b|(?-i:\b[A-Z]{0,4}RTC\b|\bDTC\b|\bBMTC\b)\s+(?:bus|buses)\b|\brailways?\s+(?:station|stations|track|tracks|coach|coaches|bogie|bogies|engine|engines|line|lines|signal|signals|gate|gates|train|trains|bus)\b|\btrain\s+coach(?:es)?\b|\bpolice\s+(?:station|stations|vehicle|vehicles|jeeps?|vans?|outposts?|post|chowki|barricades?)\b|\bmunicipal\s+(?:building|buildings|office|offices|bus|buses|vehicle|vehicles)\b|\bpanchayat\s+(?:office|offices|building|buildings|bhawan|bhavan)\b|\btehsil(?:dar'?s?)?\s+(?:office|offices|building)\b|\bcollector'?s?\s+office\b|\bcollectorate\b|\bpost\s+office\b|\bcourt\s+(?:building|buildings|premises|complex)\b|\bbus\s+(?:stand|stands|depot|station|shelter|stop)\b|\bmetro\s+(?:train|trains|station|stations|coach|coaches)\b|\btoll\s+(?:plaza|booth|gate)\b|\bstreet\s*lights?\b|\bsignal\s+lights?\b|\btraffic\s+(?:signals?|lights?)\b|\belectricity\s+(?:poles?|transformers?|substation|lines?)\b|\bration\s+shop\b)|(?:\bpublic\s+(?:building|buildings|transport|vehicle|vehicles|bus|buses|utility|utilities|asset|assets|toilets?|library|park)\b|\b(?:government|govt\.?|state)\s+(?:building|buildings|office|offices|vehicle|vehicles|bus|buses|school|schools|hospital|hospitals|college|colleges|premises|asset|assets|establishment|establishments|transport|jeeps?|guest\s+house)\b|\b(?:state\s+transport|roadways|road\s+transport)\b|(?-i:\b[A-Z]{0,4}RTC\b|\bDTC\b|\bBMTC\b)\s+(?:bus|buses)\b|\brailways?\s+(?:station|stations|track|tracks|coach|coaches|bogie|bogies|engine|engines|line|lines|signal|signals|gate|gates|train|trains|bus)\b|\btrain\s+coach(?:es)?\b|\bpolice\s+(?:station|stations|vehicle|vehicles|jeeps?|vans?|outposts?|post|chowki|barricades?)\b|\bmunicipal\s+(?:building|buildings|office|offices|bus|buses|vehicle|vehicles)\b|\bpanchayat\s+(?:office|offices|building|buildings|bhawan|bhavan)\b|\btehsil(?:dar'?s?)?\s+(?:office|offices|building)\b|\bcollector'?s?\s+office\b|\bcollectorate\b|\bpost\s+office\b|\bcourt\s+(?:building|buildings|premises|complex)\b|\bbus\s+(?:stand|stands|depot|station|shelter|stop)\b|\bmetro\s+(?:train|trains|station|stations|coach|coaches)\b|\btoll\s+(?:plaza|booth|gate)\b|\bstreet\s*lights?\b|\bsignal\s+lights?\b|\btraffic\s+(?:signals?|lights?)\b|\belectricity\s+(?:poles?|transformers?|substation|lines?)\b|\bration\s+shop\b)\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,3}?(?:was|were|got|gets|is|are|been|being)\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,2}?(?:(?:\bset(?:ting|s)?\s+fire\b|\btorch\w*|\barson\w*|\bburn\w*|\bgutted\b|\bvandali[sz]\w*|\bransack\w*|\bsmash\w*|\bstoned\b|\bstone[- ]?pelt\w*|\bset(?:ting|s)?\s+ablaze\b|\b(?:threw|thrown|throwing|throw|throws|pelt\w*|hurl\w*)\s+(?:\w+\s+){0,2}?(?:stones?|bricks?|petrol\s+bombs?|bottles?)\b|\bpetrol\s+bombs?\b)|\b(?:break(?:ing|s)?|broke|broken)\s+(?:\w+\s+){0,3}?(?:windows?|windscreens?|windshields?|glass|doors?|gates?|furniture|signals?|lights?|barricades?)\b))</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Prevention of Damage to Public Property Act, 1984</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>'set a ... on fire / ablaze' where the thing is one of the public things above</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Needed because the thing sits inside the verb phrase.</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>\bset(?:ting|s)?\s+(?:[\w']+\s+){0,4}?(?:(?:\bpublic\s+(?:building|buildings|transport|vehicle|vehicles|bus|buses|utility|utilities|asset|assets|toilets?|library|park)\b|\b(?:government|govt\.?|state)\s+(?:building|buildings|office|offices|vehicle|vehicles|bus|buses|school|schools|hospital|hospitals|college|colleges|premises|asset|assets|establishment|establishments|transport|jeeps?|guest\s+house)\b|\b(?:state\s+transport|roadways|road\s+transport)\b|(?-i:\b[A-Z]{0,4}RTC\b|\bDTC\b|\bBMTC\b)\s+(?:bus|buses)\b|\brailways?\s+(?:station|stations|track|tracks|coach|coaches|bogie|bogies|engine|engines|line|lines|signal|signals|gate|gates|train|trains|bus)\b|\btrain\s+coach(?:es)?\b|\bpolice\s+(?:station|stations|vehicle|vehicles|jeeps?|vans?|outposts?|post|chowki|barricades?)\b|\bmunicipal\s+(?:building|buildings|office|offices|bus|buses|vehicle|vehicles)\b|\bpanchayat\s+(?:office|offices|building|buildings|bhawan|bhavan)\b|\btehsil(?:dar'?s?)?\s+(?:office|offices|building)\b|\bcollector'?s?\s+office\b|\bcollectorate\b|\bpost\s+office\b|\bcourt\s+(?:building|buildings|premises|complex)\b|\bbus\s+(?:stand|stands|depot|station|shelter|stop)\b|\bmetro\s+(?:train|trains|station|stations|coach|coaches)\b|\btoll\s+(?:plaza|booth|gate)\b|\bstreet\s*lights?\b|\bsignal\s+lights?\b|\btraffic\s+(?:signals?|lights?)\b|\belectricity\s+(?:poles?|transformers?|substation|lines?)\b|\bration\s+shop\b)).{0,30}?\b(?:on\s+fire|ablaze|alight)\b</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Prevention of Damage to Public Property Act, 1984</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>'broke / breaking the ...' with the public thing itself as the object (signal lights, street lights ...)</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Added after the harder question set missed 'breaking the signal lights and barricades at the junction'.</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>\b(?:break(?:ing|s)?|broke|broken)\s+(?:(?:the|a|an|all|some|several|many|two|three|their|its)\s+){0,2}(?:(?:\bpublic\s+(?:building|buildings|transport|vehicle|vehicles|bus|buses|utility|utilities|asset|assets|toilets?|library|park)\b|\b(?:government|govt\.?|state)\s+(?:building|buildings|office|offices|vehicle|vehicles|bus|buses|school|schools|hospital|hospitals|college|colleges|premises|asset|assets|establishment|establishments|transport|jeeps?|guest\s+house)\b|\b(?:state\s+transport|roadways|road\s+transport)\b|(?-i:\b[A-Z]{0,4}RTC\b|\bDTC\b|\bBMTC\b)\s+(?:bus|buses)\b|\brailways?\s+(?:station|stations|track|tracks|coach|coaches|bogie|bogies|engine|engines|line|lines|signal|signals|gate|gates|train|trains|bus)\b|\btrain\s+coach(?:es)?\b|\bpolice\s+(?:station|stations|vehicle|vehicles|jeeps?|vans?|outposts?|post|chowki|barricades?)\b|\bmunicipal\s+(?:building|buildings|office|offices|bus|buses|vehicle|vehicles)\b|\bpanchayat\s+(?:office|offices|building|buildings|bhawan|bhavan)\b|\btehsil(?:dar'?s?)?\s+(?:office|offices|building)\b|\bcollector'?s?\s+office\b|\bcollectorate\b|\bpost\s+office\b|\bcourt\s+(?:building|buildings|premises|complex)\b|\bbus\s+(?:stand|stands|depot|station|shelter|stop)\b|\bmetro\s+(?:train|trains|station|stations|coach|coaches)\b|\btoll\s+(?:plaza|booth|gate)\b|\bstreet\s*lights?\b|\bsignal\s+lights?\b|\btraffic\s+(?:signals?|lights?)\b|\belectricity\s+(?:poles?|transformers?|substation|lines?)\b|\bration\s+shop\b))</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Prevention of Damage to Public Property Act, 1984</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>any damage word, including the milder 'damaged' and 'destroyed', with one of the public things above, AND a protest word within 120 characters (protest, riot, bandh, hartal, shutdown, agitation, demonstration, dharna, strike, mob, clash, rally, crowd, lathi-charge, rasta roko, rail roko, road blockade, 'blocked the highway' ...)</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>The workbook's note: 'do not apply its boost to private-property damage or a protest mention without a public-property damage cue'. Both cues are needed. 'Shutdown' and 'blocked the highway' were added after the harder question set.</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:(?:(?:(?:\bset(?:ting|s)?\s+fire\b|\btorch\w*|\barson\w*|\bburn\w*|\bgutted\b|\bvandali[sz]\w*|\bransack\w*|\bsmash\w*|\bstoned\b|\bstone[- ]?pelt\w*|\bset(?:ting|s)?\s+ablaze\b|\b(?:threw|thrown|throwing|throw|throws|pelt\w*|hurl\w*)\s+(?:\w+\s+){0,2}?(?:stones?|bricks?|petrol\s+bombs?|bottles?)\b|\bpetrol\s+bombs?\b)|\b(?:break(?:ing|s)?|broke|broken)\s+(?:\w+\s+){0,3}?(?:windows?|windscreens?|windshields?|glass|doors?|gates?|furniture|signals?|lights?|barricades?)\b|(?:\bdamag\w+|\bdestr(?:oy\w*|uction|uctive)\b|\bwreck\w*|\bruin\w*))\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,5}?(?:\bpublic\s+(?:building|buildings|transport|vehicle|vehicles|bus|buses|utility|utilities|asset|assets|toilets?|library|park)\b|\b(?:government|govt\.?|state)\s+(?:building|buildings|office|offices|vehicle|vehicles|bus|buses|school|schools|hospital|hospitals|college|colleges|premises|asset|assets|establishment|establishments|transport|jeeps?|guest\s+house)\b|\b(?:state\s+transport|roadways|road\s+transport)\b|(?-i:\b[A-Z]{0,4}RTC\b|\bDTC\b|\bBMTC\b)\s+(?:bus|buses)\b|\brailways?\s+(?:station|stations|track|tracks|coach|coaches|bogie|bogies|engine|engines|line|lines|signal|signals|gate|gates|train|trains|bus)\b|\btrain\s+coach(?:es)?\b|\bpolice\s+(?:station|stations|vehicle|vehicles|jeeps?|vans?|outposts?|post|chowki|barricades?)\b|\bmunicipal\s+(?:building|buildings|office|offices|bus|buses|vehicle|vehicles)\b|\bpanchayat\s+(?:office|offices|building|buildings|bhawan|bhavan)\b|\btehsil(?:dar'?s?)?\s+(?:office|offices|building)\b|\bcollector'?s?\s+office\b|\bcollectorate\b|\bpost\s+office\b|\bcourt\s+(?:building|buildings|premises|complex)\b|\bbus\s+(?:stand|stands|depot|station|shelter|stop)\b|\bmetro\s+(?:train|trains|station|stations|coach|coaches)\b|\btoll\s+(?:plaza|booth|gate)\b|\bstreet\s*lights?\b|\bsignal\s+lights?\b|\btraffic\s+(?:signals?|lights?)\b|\belectricity\s+(?:poles?|transformers?|substation|lines?)\b|\bration\s+shop\b)|(?:\bpublic\s+(?:building|buildings|transport|vehicle|vehicles|bus|buses|utility|utilities|asset|assets|toilets?|library|park)\b|\b(?:government|govt\.?|state)\s+(?:building|buildings|office|offices|vehicle|vehicles|bus|buses|school|schools|hospital|hospitals|college|colleges|premises|asset|assets|establishment|establishments|transport|jeeps?|guest\s+house)\b|\b(?:state\s+transport|roadways|road\s+transport)\b|(?-i:\b[A-Z]{0,4}RTC\b|\bDTC\b|\bBMTC\b)\s+(?:bus|buses)\b|\brailways?\s+(?:station|stations|track|tracks|coach|coaches|bogie|bogies|engine|engines|line|lines|signal|signals|gate|gates|train|trains|bus)\b|\btrain\s+coach(?:es)?\b|\bpolice\s+(?:station|stations|vehicle|vehicles|jeeps?|vans?|outposts?|post|chowki|barricades?)\b|\bmunicipal\s+(?:building|buildings|office|offices|bus|buses|vehicle|vehicles)\b|\bpanchayat\s+(?:office|offices|building|buildings|bhawan|bhavan)\b|\btehsil(?:dar'?s?)?\s+(?:office|offices|building)\b|\bcollector'?s?\s+office\b|\bcollectorate\b|\bpost\s+office\b|\bcourt\s+(?:building|buildings|premises|complex)\b|\bbus\s+(?:stand|stands|depot|station|shelter|stop)\b|\bmetro\s+(?:train|trains|station|stations|coach|coaches)\b|\btoll\s+(?:plaza|booth|gate)\b|\bstreet\s*lights?\b|\bsignal\s+lights?\b|\btraffic\s+(?:signals?|lights?)\b|\belectricity\s+(?:poles?|transformers?|substation|lines?)\b|\bration\s+shop\b)\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,3}?(?:was|were|got|gets|is|are|been|being)\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,2}?(?:(?:\bset(?:ting|s)?\s+fire\b|\btorch\w*|\barson\w*|\bburn\w*|\bgutted\b|\bvandali[sz]\w*|\bransack\w*|\bsmash\w*|\bstoned\b|\bstone[- ]?pelt\w*|\bset(?:ting|s)?\s+ablaze\b|\b(?:threw|thrown|throwing|throw|throws|pelt\w*|hurl\w*)\s+(?:\w+\s+){0,2}?(?:stones?|bricks?|petrol\s+bombs?|bottles?)\b|\bpetrol\s+bombs?\b)|\b(?:break(?:ing|s)?|broke|broken)\s+(?:\w+\s+){0,3}?(?:windows?|windscreens?|windshields?|glass|doors?|gates?|furniture|signals?|lights?|barricades?)\b|(?:\bdamag\w+|\bdestr(?:oy\w*|uction|uctive)\b|\bwreck\w*|\bruin\w*)))).{0,120}(?:\b(?:protest\w*|riot\w*|bandh|bundh|hartal|shutdown|agitat\w+|demonstrat\w+|dharna|strikes?|striking|strikers?|mob|mobs|violen\w+|clash\w*|unrest|rasta[- ]?roko|rail[- ]?roko|chakka[- ]?jam|morcha|procession|rally|rallies|lathi[- ]?charge|curfew|unruly|crowd|crowds|rioters?|agitators?|blockade|andolan|block(?:ed|ing|s)?\s+(?:the\s+)?(?:road|roads|highway|highways|rail|railway|track|tracks|traffic))\b)|(?:\b(?:protest\w*|riot\w*|bandh|bundh|hartal|shutdown|agitat\w+|demonstrat\w+|dharna|strikes?|striking|strikers?|mob|mobs|violen\w+|clash\w*|unrest|rasta[- ]?roko|rail[- ]?roko|chakka[- ]?jam|morcha|procession|rally|rallies|lathi[- ]?charge|curfew|unruly|crowd|crowds|rioters?|agitators?|blockade|andolan|block(?:ed|ing|s)?\s+(?:the\s+)?(?:road|roads|highway|highways|rail|railway|track|tracks|traffic))\b).{0,120}(?:(?:(?:(?:\bset(?:ting|s)?\s+fire\b|\btorch\w*|\barson\w*|\bburn\w*|\bgutted\b|\bvandali[sz]\w*|\bransack\w*|\bsmash\w*|\bstoned\b|\bstone[- ]?pelt\w*|\bset(?:ting|s)?\s+ablaze\b|\b(?:threw|thrown|throwing|throw|throws|pelt\w*|hurl\w*)\s+(?:\w+\s+){0,2}?(?:stones?|bricks?|petrol\s+bombs?|bottles?)\b|\bpetrol\s+bombs?\b)|\b(?:break(?:ing|s)?|broke|broken)\s+(?:\w+\s+){0,3}?(?:windows?|windscreens?|windshields?|glass|doors?|gates?|furniture|signals?|lights?|barricades?)\b|(?:\bdamag\w+|\bdestr(?:oy\w*|uction|uctive)\b|\bwreck\w*|\bruin\w*))\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,5}?(?:\bpublic\s+(?:building|buildings|transport|vehicle|vehicles|bus|buses|utility|utilities|asset|assets|toilets?|library|park)\b|\b(?:government|govt\.?|state)\s+(?:building|buildings|office|offices|vehicle|vehicles|bus|buses|school|schools|hospital|hospitals|college|colleges|premises|asset|assets|establishment|establishments|transport|jeeps?|guest\s+house)\b|\b(?:state\s+transport|roadways|road\s+transport)\b|(?-i:\b[A-Z]{0,4}RTC\b|\bDTC\b|\bBMTC\b)\s+(?:bus|buses)\b|\brailways?\s+(?:station|stations|track|tracks|coach|coaches|bogie|bogies|engine|engines|line|lines|signal|signals|gate|gates|train|trains|bus)\b|\btrain\s+coach(?:es)?\b|\bpolice\s+(?:station|stations|vehicle|vehicles|jeeps?|vans?|outposts?|post|chowki|barricades?)\b|\bmunicipal\s+(?:building|buildings|office|offices|bus|buses|vehicle|vehicles)\b|\bpanchayat\s+(?:office|offices|building|buildings|bhawan|bhavan)\b|\btehsil(?:dar'?s?)?\s+(?:office|offices|building)\b|\bcollector'?s?\s+office\b|\bcollectorate\b|\bpost\s+office\b|\bcourt\s+(?:building|buildings|premises|complex)\b|\bbus\s+(?:stand|stands|depot|station|shelter|stop)\b|\bmetro\s+(?:train|trains|station|stations|coach|coaches)\b|\btoll\s+(?:plaza|booth|gate)\b|\bstreet\s*lights?\b|\bsignal\s+lights?\b|\btraffic\s+(?:signals?|lights?)\b|\belectricity\s+(?:poles?|transformers?|substation|lines?)\b|\bration\s+shop\b)|(?:\bpublic\s+(?:building|buildings|transport|vehicle|vehicles|bus|buses|utility|utilities|asset|assets|toilets?|library|park)\b|\b(?:government|govt\.?|state)\s+(?:building|buildings|office|offices|vehicle|vehicles|bus|buses|school|schools|hospital|hospitals|college|colleges|premises|asset|assets|establishment|establishments|transport|jeeps?|guest\s+house)\b|\b(?:state\s+transport|roadways|road\s+transport)\b|(?-i:\b[A-Z]{0,4}RTC\b|\bDTC\b|\bBMTC\b)\s+(?:bus|buses)\b|\brailways?\s+(?:station|stations|track|tracks|coach|coaches|bogie|bogies|engine|engines|line|lines|signal|signals|gate|gates|train|trains|bus)\b|\btrain\s+coach(?:es)?\b|\bpolice\s+(?:station|stations|vehicle|vehicles|jeeps?|vans?|outposts?|post|chowki|barricades?)\b|\bmunicipal\s+(?:building|buildings|office|offices|bus|buses|vehicle|vehicles)\b|\bpanchayat\s+(?:office|offices|building|buildings|bhawan|bhavan)\b|\btehsil(?:dar'?s?)?\s+(?:office|offices|building)\b|\bcollector'?s?\s+office\b|\bcollectorate\b|\bpost\s+office\b|\bcourt\s+(?:building|buildings|premises|complex)\b|\bbus\s+(?:stand|stands|depot|station|shelter|stop)\b|\bmetro\s+(?:train|trains|station|stations|coach|coaches)\b|\btoll\s+(?:plaza|booth|gate)\b|\bstreet\s*lights?\b|\bsignal\s+lights?\b|\btraffic\s+(?:signals?|lights?)\b|\belectricity\s+(?:poles?|transformers?|substation|lines?)\b|\bration\s+shop\b)\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,3}?(?:was|were|got|gets|is|are|been|being)\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,2}?(?:(?:\bset(?:ting|s)?\s+fire\b|\btorch\w*|\barson\w*|\bburn\w*|\bgutted\b|\bvandali[sz]\w*|\bransack\w*|\bsmash\w*|\bstoned\b|\bstone[- ]?pelt\w*|\bset(?:ting|s)?\s+ablaze\b|\b(?:threw|thrown|throwing|throw|throws|pelt\w*|hurl\w*)\s+(?:\w+\s+){0,2}?(?:stones?|bricks?|petrol\s+bombs?|bottles?)\b|\bpetrol\s+bombs?\b)|\b(?:break(?:ing|s)?|broke|broken)\s+(?:\w+\s+){0,3}?(?:windows?|windscreens?|windshields?|glass|doors?|gates?|furniture|signals?|lights?|barricades?)\b|(?:\bdamag\w+|\bdestr(?:oy\w*|uction|uctive)\b|\bwreck\w*|\bruin\w*)))))</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Prevention of Damage to Public Property Act, 1984</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>the same for a plain bus, train, tram, metro or railway (which could be private), only with a protest word</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>A bare 'bus' is not necessarily public property, so the protest word is what makes it count.</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:(?:(?:(?:\bset(?:ting|s)?\s+fire\b|\btorch\w*|\barson\w*|\bburn\w*|\bgutted\b|\bvandali[sz]\w*|\bransack\w*|\bsmash\w*|\bstoned\b|\bstone[- ]?pelt\w*|\bset(?:ting|s)?\s+ablaze\b|\b(?:threw|thrown|throwing|throw|throws|pelt\w*|hurl\w*)\s+(?:\w+\s+){0,2}?(?:stones?|bricks?|petrol\s+bombs?|bottles?)\b|\bpetrol\s+bombs?\b)|\b(?:break(?:ing|s)?|broke|broken)\s+(?:\w+\s+){0,3}?(?:windows?|windscreens?|windshields?|glass|doors?|gates?|furniture|signals?|lights?|barricades?)\b|(?:\bdamag\w+|\bdestr(?:oy\w*|uction|uctive)\b|\bwreck\w*|\bruin\w*))\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,3}?\b(?:bus|buses|train|trains|tram|trams|metro|railway|railways)\b|\b(?:bus|buses|train|trains|tram|trams|metro|railway|railways)\b\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,3}?(?:was|were|got|gets|is|are|been|being)\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,2}?(?:(?:\bset(?:ting|s)?\s+fire\b|\btorch\w*|\barson\w*|\bburn\w*|\bgutted\b|\bvandali[sz]\w*|\bransack\w*|\bsmash\w*|\bstoned\b|\bstone[- ]?pelt\w*|\bset(?:ting|s)?\s+ablaze\b|\b(?:threw|thrown|throwing|throw|throws|pelt\w*|hurl\w*)\s+(?:\w+\s+){0,2}?(?:stones?|bricks?|petrol\s+bombs?|bottles?)\b|\bpetrol\s+bombs?\b)|\b(?:break(?:ing|s)?|broke|broken)\s+(?:\w+\s+){0,3}?(?:windows?|windscreens?|windshields?|glass|doors?|gates?|furniture|signals?|lights?|barricades?)\b|(?:\bdamag\w+|\bdestr(?:oy\w*|uction|uctive)\b|\bwreck\w*|\bruin\w*)))).{0,120}(?:\b(?:protest\w*|riot\w*|bandh|bundh|hartal|shutdown|agitat\w+|demonstrat\w+|dharna|strikes?|striking|strikers?|mob|mobs|violen\w+|clash\w*|unrest|rasta[- ]?roko|rail[- ]?roko|chakka[- ]?jam|morcha|procession|rally|rallies|lathi[- ]?charge|curfew|unruly|crowd|crowds|rioters?|agitators?|blockade|andolan|block(?:ed|ing|s)?\s+(?:the\s+)?(?:road|roads|highway|highways|rail|railway|track|tracks|traffic))\b)|(?:\b(?:protest\w*|riot\w*|bandh|bundh|hartal|shutdown|agitat\w+|demonstrat\w+|dharna|strikes?|striking|strikers?|mob|mobs|violen\w+|clash\w*|unrest|rasta[- ]?roko|rail[- ]?roko|chakka[- ]?jam|morcha|procession|rally|rallies|lathi[- ]?charge|curfew|unruly|crowd|crowds|rioters?|agitators?|blockade|andolan|block(?:ed|ing|s)?\s+(?:the\s+)?(?:road|roads|highway|highways|rail|railway|track|tracks|traffic))\b).{0,120}(?:(?:(?:(?:\bset(?:ting|s)?\s+fire\b|\btorch\w*|\barson\w*|\bburn\w*|\bgutted\b|\bvandali[sz]\w*|\bransack\w*|\bsmash\w*|\bstoned\b|\bstone[- ]?pelt\w*|\bset(?:ting|s)?\s+ablaze\b|\b(?:threw|thrown|throwing|throw|throws|pelt\w*|hurl\w*)\s+(?:\w+\s+){0,2}?(?:stones?|bricks?|petrol\s+bombs?|bottles?)\b|\bpetrol\s+bombs?\b)|\b(?:break(?:ing|s)?|broke|broken)\s+(?:\w+\s+){0,3}?(?:windows?|windscreens?|windshields?|glass|doors?|gates?|furniture|signals?|lights?|barricades?)\b|(?:\bdamag\w+|\bdestr(?:oy\w*|uction|uctive)\b|\bwreck\w*|\bruin\w*))\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,3}?\b(?:bus|buses|train|trains|tram|trams|metro|railway|railways)\b|\b(?:bus|buses|train|trains|tram|trams|metro|railway|railways)\b\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,3}?(?:was|were|got|gets|is|are|been|being)\s+(?:(?!(?:went|go|goes|going|gone|visited|reached|complain\w*|report\w*|lodg\w+|filed|registered|called|brought|taken|took)\b)[\w'’,-]+\s+){0,2}?(?:(?:\bset(?:ting|s)?\s+fire\b|\btorch\w*|\barson\w*|\bburn\w*|\bgutted\b|\bvandali[sz]\w*|\bransack\w*|\bsmash\w*|\bstoned\b|\bstone[- ]?pelt\w*|\bset(?:ting|s)?\s+ablaze\b|\b(?:threw|thrown|throwing|throw|throws|pelt\w*|hurl\w*)\s+(?:\w+\s+){0,2}?(?:stones?|bricks?|petrol\s+bombs?|bottles?)\b|\bpetrol\s+bombs?\b)|\b(?:break(?:ing|s)?|broke|broken)\s+(?:\w+\s+){0,3}?(?:windows?|windscreens?|windshields?|glass|doors?|gates?|furniture|signals?|lights?|barricades?)\b|(?:\bdamag\w+|\bdestr(?:oy\w*|uction|uctive)\b|\bwreck\w*|\bruin\w*)))))</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Prevention of Damage to Public Property Act, 1984</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>'a bus was set on fire' and the like, for a plain bus or train, only with a protest word</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Same.</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>(?:(?:\bset(?:ting|s)?\s+(?:[\w']+\s+){0,4}?(?:\b(?:bus|buses|train|trains|tram|trams|metro|railway|railways)\b).{0,30}?\b(?:on\s+fire|ablaze|alight)\b).{0,120}(?:\b(?:protest\w*|riot\w*|bandh|bundh|hartal|shutdown|agitat\w+|demonstrat\w+|dharna|strikes?|striking|strikers?|mob|mobs|violen\w+|clash\w*|unrest|rasta[- ]?roko|rail[- ]?roko|chakka[- ]?jam|morcha|procession|rally|rallies|lathi[- ]?charge|curfew|unruly|crowd|crowds|rioters?|agitators?|blockade|andolan|block(?:ed|ing|s)?\s+(?:the\s+)?(?:road|roads|highway|highways|rail|railway|track|tracks|traffic))\b)|(?:\b(?:protest\w*|riot\w*|bandh|bundh|hartal|shutdown|agitat\w+|demonstrat\w+|dharna|strikes?|striking|strikers?|mob|mobs|violen\w+|clash\w*|unrest|rasta[- ]?roko|rail[- ]?roko|chakka[- ]?jam|morcha|procession|rally|rallies|lathi[- ]?charge|curfew|unruly|crowd|crowds|rioters?|agitators?|blockade|andolan|block(?:ed|ing|s)?\s+(?:the\s+)?(?:road|roads|highway|highways|rail|railway|track|tracks|traffic))\b).{0,120}(?:\bset(?:ting|s)?\s+(?:[\w']+\s+){0,4}?(?:\b(?:bus|buses|train|trains|tram|trams|metro|railway|railways)\b).{0,30}?\b(?:on\s+fire|ablaze|alight)\b))</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2841,7 +3641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2897,42 +3697,86 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Protection of Children from Sexual Offences Act, 2012 (POCSO)</t>
+          <t>Muslim Women (Protection of Rights on Marriage) Act, 2019</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Workbook, same words</t>
+          <t>Mine (not in the workbook)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Does NOT fire if the question contains an adult age (18+ year old, aged 18+) or any of: adult, boss, employer, colleague, workplace.</t>
+          <t>Two guards, each lifted by a sign that talaq WAS pronounced instantly. (1) Switched OFF if the question has talaq-e-hasan or talaq-e-ahsan (not instantaneous, so not covered by the Act's section 2(c) as written), or 'Protection of Rights on Divorce', or '1986' (the other Muslim Women Act), UNLESS it also says biddat, triple, instant, at once, in one go, a single sitting or breath, immediate or irrevocable. (2) Switched OFF if the question is a threat or a future ('talaq if I ...', 'will give', 'would say', 'going to give', 'threatened', 'warned me') UNLESS it also says thrice, three times, teen baar, biddat, triple, instant, already, 'has given', pronounced, 'gave me'.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Workbook N2 exclusion, same words.</t>
+          <t>Mine. Guard (1) comes from the Revised Trigger Map's note that not every talaq is covered. Guard (2) was added after the harder question set raised the Act on 'he said he will give me talaq if I speak to my parents on the phone'.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Prevention of Damage to Public Property Act, 1984</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Mine (not in the workbook)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Two guards, each lifted by a protest, riot, bandh, mob, clash or similar word. (1) Switched OFF if the question has an accident, collision, short circuit, caught fire, 'fire broke out', gas leak, lightning, heavy rain, flood, storm, earthquake or cyclone. (2) Switched OFF if the question is about a burn injury ('burn injuries', 'burn victim', 'suffered burns', 'burnt his hand', 'first-degree').</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Mine. Guard (2) was added after the harder question set raised the Act on 'my child suffered burn injuries and was admitted to a government hospital'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Protection of Children from Sexual Offences Act, 2012 (POCSO)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Workbook, same words</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Does NOT fire if the question contains an adult age (18+ year old, aged 18+) or any of: adult, boss, employer, colleague, workplace.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Workbook N2 exclusion, same words.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>Juvenile Justice (Care and Protection of Children) Act, 2015</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Workbook, same words</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Does NOT fire if the question contains sexual..., molest..., rape... or pornograph... (a sexual offence against a child is POCSO's).</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Workbook N2 exclusion, same words.</t>
         </is>
@@ -5430,7 +6274,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>No word pass. All seven are in the Directory (names/phrases) and can be chosen by the AI pass. The Child Marriage, Civil Rights, Public Property and Muslim Women Acts were added to the Directory on 2026-10-17 with names and phrases drawn from the workbook's own strong terms; their false-positive notes (child marriage also arises under POCSO and personal law; the PCR Act is not the SC/ST Act; triple talaq also arises in constitutional discussion) are why they get no word pass.</t>
+          <t>All seven are in the Directory (names/phrases) and can be chosen by the AI pass. The Child Marriage, Civil Rights, Public Property and Muslim Women Acts were added to the Directory on 2026-10-17 with names and phrases drawn from the workbook's own strong terms. The Muslim Women and Public Property Acts then got a word pass of their own (same day, owner's go); the Child Marriage and Civil Rights Acts did NOT, because the workbook's false-positive notes (child marriage also arises under POCSO and personal law; the PCR Act overlaps the SC/ST Act) mean a word pass would often raise the wrong one of two overlapping Acts.</t>
         </is>
       </c>
     </row>

</xml_diff>